<commit_message>
Make the demo workbook match how 002 was recorded
The generator reserved column O for the array formula, expecting the live list
to appear beside the typed one. Josh put the array in M5 itself, replacing the
typed list in place -- which is the better demo, because the list the viewer has
been looking at is the one that becomes self-maintaining. So the workbook
follows the recording rather than the reverse, and nothing is reserved in O.

The concrete fix is the border. It covered exactly the six typed rows, so when
=SORT(UNIQUE(...)) spilled seven values the seventh sat outside the box -- the
cosmetic wart Josh narrated noticing at 1:33 in the raw take, and the last thing
on screen before the recap card. Three blank-but-bordered rows now sit under the
list, so the box still fits when it grows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/two-minute-training-tuesday/episodes/001-excel-dynamic-arrays/demo-workbook-solved.xlsx
+++ b/two-minute-training-tuesday/episodes/001-excel-dynamic-arrays/demo-workbook-solved.xlsx
@@ -11207,7 +11207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M10"/>
+  <dimension ref="B1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -11326,6 +11326,15 @@
           <t>Shipping</t>
         </is>
       </c>
+    </row>
+    <row r="11">
+      <c r="M11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="M12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="M13" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>